<commit_message>
data: sync PC-server-0148 2026-09-24 21:39
</commit_message>
<xml_diff>
--- a/data/去哪儿xss.xlsx
+++ b/data/去哪儿xss.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE171"/>
+  <dimension ref="A1:AE175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20978,11 +20978,7 @@
           <t>*</t>
         </is>
       </c>
-      <c r="N171" t="inlineStr">
-        <is>
-          <t>2026-09-24 08:10:27</t>
-        </is>
-      </c>
+      <c r="N171" t="inlineStr"/>
       <c r="O171" t="n">
         <v>-2</v>
       </c>
@@ -21027,10 +21023,8 @@
           <t>2026-09-24 16:40:27</t>
         </is>
       </c>
-      <c r="AA171" t="inlineStr">
-        <is>
-          <t>2919569830</t>
-        </is>
+      <c r="AA171" t="n">
+        <v>2919569830</v>
       </c>
       <c r="AB171" t="inlineStr">
         <is>
@@ -21048,6 +21042,496 @@
         </is>
       </c>
       <c r="AE171" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>2919596077</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>xss.trade.qunar.com</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>1</v>
+      </c>
+      <c r="D172" t="n">
+        <v>0</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>0</v>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>1970-01-01</t>
+        </is>
+      </c>
+      <c r="K172" t="n">
+        <v>-62170185600000</v>
+      </c>
+      <c r="L172" t="inlineStr"/>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="N172" t="inlineStr"/>
+      <c r="O172" t="n">
+        <v>-2</v>
+      </c>
+      <c r="P172" t="inlineStr"/>
+      <c r="Q172" t="n">
+        <v>1</v>
+      </c>
+      <c r="R172" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="S172" t="inlineStr">
+        <is>
+          <t>2026-09-24 17:58:28</t>
+        </is>
+      </c>
+      <c r="T172" t="n">
+        <v>1</v>
+      </c>
+      <c r="U172" t="n">
+        <v>0</v>
+      </c>
+      <c r="V172" t="n">
+        <v>0</v>
+      </c>
+      <c r="W172" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="X172" t="inlineStr">
+        <is>
+          <t>AFARE</t>
+        </is>
+      </c>
+      <c r="Y172" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z172" t="inlineStr">
+        <is>
+          <t>2026-09-24 18:28:28</t>
+        </is>
+      </c>
+      <c r="AA172" t="n">
+        <v>2919596077</v>
+      </c>
+      <c r="AB172" t="inlineStr">
+        <is>
+          <t>Rid:domestic_5001</t>
+        </is>
+      </c>
+      <c r="AC172" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AD172" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AE172" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>2919604306</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>xss.trade.qunar.com</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>1</v>
+      </c>
+      <c r="D173" t="n">
+        <v>0</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>0</v>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>1970-01-01</t>
+        </is>
+      </c>
+      <c r="K173" t="n">
+        <v>-62170185600000</v>
+      </c>
+      <c r="L173" t="inlineStr"/>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="N173" t="inlineStr"/>
+      <c r="O173" t="n">
+        <v>-2</v>
+      </c>
+      <c r="P173" t="inlineStr"/>
+      <c r="Q173" t="n">
+        <v>1</v>
+      </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="S173" t="inlineStr">
+        <is>
+          <t>2026-09-24 18:35:00</t>
+        </is>
+      </c>
+      <c r="T173" t="n">
+        <v>1</v>
+      </c>
+      <c r="U173" t="n">
+        <v>0</v>
+      </c>
+      <c r="V173" t="n">
+        <v>0</v>
+      </c>
+      <c r="W173" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="X173" t="inlineStr">
+        <is>
+          <t>AFARE</t>
+        </is>
+      </c>
+      <c r="Y173" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z173" t="inlineStr">
+        <is>
+          <t>2026-09-24 18:50:00</t>
+        </is>
+      </c>
+      <c r="AA173" t="n">
+        <v>2919604306</v>
+      </c>
+      <c r="AB173" t="inlineStr">
+        <is>
+          <t>Rid:domestic_4012</t>
+        </is>
+      </c>
+      <c r="AC173" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AD173" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AE173" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>2919616354</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>xss.trade.qunar.com</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>1</v>
+      </c>
+      <c r="D174" t="n">
+        <v>0</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>0</v>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>1970-01-01</t>
+        </is>
+      </c>
+      <c r="K174" t="n">
+        <v>-62170185600000</v>
+      </c>
+      <c r="L174" t="inlineStr"/>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="N174" t="inlineStr"/>
+      <c r="O174" t="n">
+        <v>-2</v>
+      </c>
+      <c r="P174" t="inlineStr"/>
+      <c r="Q174" t="n">
+        <v>1</v>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="S174" t="inlineStr">
+        <is>
+          <t>2026-09-24 19:30:00</t>
+        </is>
+      </c>
+      <c r="T174" t="n">
+        <v>1</v>
+      </c>
+      <c r="U174" t="n">
+        <v>0</v>
+      </c>
+      <c r="V174" t="n">
+        <v>0</v>
+      </c>
+      <c r="W174" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="X174" t="inlineStr">
+        <is>
+          <t>AFARE</t>
+        </is>
+      </c>
+      <c r="Y174" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z174" t="inlineStr">
+        <is>
+          <t>2026-09-24 19:40:00</t>
+        </is>
+      </c>
+      <c r="AA174" t="n">
+        <v>2919616354</v>
+      </c>
+      <c r="AB174" t="inlineStr">
+        <is>
+          <t>Rid:domestic_4019</t>
+        </is>
+      </c>
+      <c r="AC174" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AD174" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AE174" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>2919620077</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>xss.trade.qunar.com</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>1</v>
+      </c>
+      <c r="D175" t="n">
+        <v>0</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I175" t="n">
+        <v>0</v>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>1970-01-01</t>
+        </is>
+      </c>
+      <c r="K175" t="n">
+        <v>-62170185600000</v>
+      </c>
+      <c r="L175" t="inlineStr"/>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>2026-09-24 11:46:15</t>
+        </is>
+      </c>
+      <c r="O175" t="n">
+        <v>-2</v>
+      </c>
+      <c r="P175" t="inlineStr"/>
+      <c r="Q175" t="n">
+        <v>1</v>
+      </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="S175" t="inlineStr">
+        <is>
+          <t>2026-09-24 19:46:15</t>
+        </is>
+      </c>
+      <c r="T175" t="n">
+        <v>1</v>
+      </c>
+      <c r="U175" t="n">
+        <v>0</v>
+      </c>
+      <c r="V175" t="n">
+        <v>0</v>
+      </c>
+      <c r="W175" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="X175" t="inlineStr">
+        <is>
+          <t>AFARE</t>
+        </is>
+      </c>
+      <c r="Y175" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z175" t="inlineStr">
+        <is>
+          <t>2026-09-24 20:16:15</t>
+        </is>
+      </c>
+      <c r="AA175" t="inlineStr">
+        <is>
+          <t>2919620077</t>
+        </is>
+      </c>
+      <c r="AB175" t="inlineStr">
+        <is>
+          <t>Rid:domestic_6001</t>
+        </is>
+      </c>
+      <c r="AC175" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AD175" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AE175" t="inlineStr">
         <is>
           <t>*</t>
         </is>

</xml_diff>

<commit_message>
data: sync PC-server-0148 2026-09-26 19:43
</commit_message>
<xml_diff>
--- a/data/去哪儿xss.xlsx
+++ b/data/去哪儿xss.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE175"/>
+  <dimension ref="A1:AE177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21462,11 +21462,7 @@
           <t>*</t>
         </is>
       </c>
-      <c r="N175" t="inlineStr">
-        <is>
-          <t>2026-09-24 11:46:15</t>
-        </is>
-      </c>
+      <c r="N175" t="inlineStr"/>
       <c r="O175" t="n">
         <v>-2</v>
       </c>
@@ -21511,10 +21507,8 @@
           <t>2026-09-24 20:16:15</t>
         </is>
       </c>
-      <c r="AA175" t="inlineStr">
-        <is>
-          <t>2919620077</t>
-        </is>
+      <c r="AA175" t="n">
+        <v>2919620077</v>
       </c>
       <c r="AB175" t="inlineStr">
         <is>
@@ -21532,6 +21526,254 @@
         </is>
       </c>
       <c r="AE175" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>2920001983</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>xss.trade.qunar.com</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>1</v>
+      </c>
+      <c r="D176" t="n">
+        <v>0</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I176" t="n">
+        <v>0</v>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>1970-01-01</t>
+        </is>
+      </c>
+      <c r="K176" t="n">
+        <v>-62170185600000</v>
+      </c>
+      <c r="L176" t="inlineStr"/>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="N176" t="inlineStr"/>
+      <c r="O176" t="n">
+        <v>-2</v>
+      </c>
+      <c r="P176" t="inlineStr"/>
+      <c r="Q176" t="n">
+        <v>1</v>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="S176" t="inlineStr">
+        <is>
+          <t>2026-09-26 16:15:00</t>
+        </is>
+      </c>
+      <c r="T176" t="n">
+        <v>1</v>
+      </c>
+      <c r="U176" t="n">
+        <v>0</v>
+      </c>
+      <c r="V176" t="n">
+        <v>0</v>
+      </c>
+      <c r="W176" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="X176" t="inlineStr">
+        <is>
+          <t>AFARE</t>
+        </is>
+      </c>
+      <c r="Y176" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z176" t="inlineStr">
+        <is>
+          <t>2026-09-26 16:25:00</t>
+        </is>
+      </c>
+      <c r="AA176" t="n">
+        <v>2920001983</v>
+      </c>
+      <c r="AB176" t="inlineStr">
+        <is>
+          <t>Rid:domestic_4013</t>
+        </is>
+      </c>
+      <c r="AC176" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AD176" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AE176" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>2920009564</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>xss.trade.qunar.com</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>1</v>
+      </c>
+      <c r="D177" t="n">
+        <v>0</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>AQ</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>0</v>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>1970-01-01</t>
+        </is>
+      </c>
+      <c r="K177" t="n">
+        <v>-62170185600000</v>
+      </c>
+      <c r="L177" t="inlineStr"/>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>2026-09-26 08:57:51</t>
+        </is>
+      </c>
+      <c r="O177" t="n">
+        <v>-2</v>
+      </c>
+      <c r="P177" t="inlineStr"/>
+      <c r="Q177" t="n">
+        <v>1</v>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="S177" t="inlineStr">
+        <is>
+          <t>2026-09-26 16:57:51</t>
+        </is>
+      </c>
+      <c r="T177" t="n">
+        <v>1</v>
+      </c>
+      <c r="U177" t="n">
+        <v>0</v>
+      </c>
+      <c r="V177" t="n">
+        <v>0</v>
+      </c>
+      <c r="W177" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="X177" t="inlineStr">
+        <is>
+          <t>AFARE</t>
+        </is>
+      </c>
+      <c r="Y177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z177" t="inlineStr">
+        <is>
+          <t>2026-09-26 17:27:51</t>
+        </is>
+      </c>
+      <c r="AA177" t="inlineStr">
+        <is>
+          <t>2920009564</t>
+        </is>
+      </c>
+      <c r="AB177" t="inlineStr">
+        <is>
+          <t>Rid:domestic_5001</t>
+        </is>
+      </c>
+      <c r="AC177" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AD177" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AE177" t="inlineStr">
         <is>
           <t>*</t>
         </is>

</xml_diff>

<commit_message>
data: sync PC-server-0148 2026-09-26 23:24
</commit_message>
<xml_diff>
--- a/data/去哪儿xss.xlsx
+++ b/data/去哪儿xss.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE177"/>
+  <dimension ref="A1:AE178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21704,11 +21704,7 @@
           <t>*</t>
         </is>
       </c>
-      <c r="N177" t="inlineStr">
-        <is>
-          <t>2026-09-26 08:57:51</t>
-        </is>
-      </c>
+      <c r="N177" t="inlineStr"/>
       <c r="O177" t="n">
         <v>-2</v>
       </c>
@@ -21753,10 +21749,8 @@
           <t>2026-09-26 17:27:51</t>
         </is>
       </c>
-      <c r="AA177" t="inlineStr">
-        <is>
-          <t>2920009564</t>
-        </is>
+      <c r="AA177" t="n">
+        <v>2920009564</v>
       </c>
       <c r="AB177" t="inlineStr">
         <is>
@@ -21774,6 +21768,133 @@
         </is>
       </c>
       <c r="AE177" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>2920057213</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>xss.trade.qunar.com</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>1</v>
+      </c>
+      <c r="D178" t="n">
+        <v>0</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>0</v>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>1970-01-01</t>
+        </is>
+      </c>
+      <c r="K178" t="n">
+        <v>-62170185600000</v>
+      </c>
+      <c r="L178" t="inlineStr"/>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:37:03</t>
+        </is>
+      </c>
+      <c r="O178" t="n">
+        <v>-2</v>
+      </c>
+      <c r="P178" t="inlineStr"/>
+      <c r="Q178" t="n">
+        <v>1</v>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="S178" t="inlineStr">
+        <is>
+          <t>2026-09-26 21:37:03</t>
+        </is>
+      </c>
+      <c r="T178" t="n">
+        <v>1</v>
+      </c>
+      <c r="U178" t="n">
+        <v>0</v>
+      </c>
+      <c r="V178" t="n">
+        <v>0</v>
+      </c>
+      <c r="W178" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="X178" t="inlineStr">
+        <is>
+          <t>AFARE</t>
+        </is>
+      </c>
+      <c r="Y178" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z178" t="inlineStr">
+        <is>
+          <t>2026-09-26 22:07:03</t>
+        </is>
+      </c>
+      <c r="AA178" t="inlineStr">
+        <is>
+          <t>2920057213</t>
+        </is>
+      </c>
+      <c r="AB178" t="inlineStr">
+        <is>
+          <t>Rid:domestic_6001</t>
+        </is>
+      </c>
+      <c r="AC178" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AD178" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AE178" t="inlineStr">
         <is>
           <t>*</t>
         </is>

</xml_diff>

<commit_message>
data: sync PC-server-0148 2026-09-29 17:55
</commit_message>
<xml_diff>
--- a/data/去哪儿xss.xlsx
+++ b/data/去哪儿xss.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE187"/>
+  <dimension ref="A1:AE190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22890,11 +22890,7 @@
           <t>*</t>
         </is>
       </c>
-      <c r="N187" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:02:30</t>
-        </is>
-      </c>
+      <c r="N187" t="inlineStr"/>
       <c r="O187" t="n">
         <v>-2</v>
       </c>
@@ -22939,10 +22935,8 @@
           <t>2026-09-28 22:32:30</t>
         </is>
       </c>
-      <c r="AA187" t="inlineStr">
-        <is>
-          <t>2920582942</t>
-        </is>
+      <c r="AA187" t="n">
+        <v>2920582942</v>
       </c>
       <c r="AB187" t="inlineStr">
         <is>
@@ -22960,6 +22954,375 @@
         </is>
       </c>
       <c r="AE187" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>2920722919</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>xss.trade.qunar.com</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>1</v>
+      </c>
+      <c r="D188" t="n">
+        <v>0</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>QW</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I188" t="n">
+        <v>0</v>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>1970-01-01</t>
+        </is>
+      </c>
+      <c r="K188" t="n">
+        <v>-62170185600000</v>
+      </c>
+      <c r="L188" t="inlineStr"/>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr"/>
+      <c r="O188" t="n">
+        <v>-2</v>
+      </c>
+      <c r="P188" t="inlineStr"/>
+      <c r="Q188" t="n">
+        <v>1</v>
+      </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="S188" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:46:56</t>
+        </is>
+      </c>
+      <c r="T188" t="n">
+        <v>1</v>
+      </c>
+      <c r="U188" t="n">
+        <v>0</v>
+      </c>
+      <c r="V188" t="n">
+        <v>0</v>
+      </c>
+      <c r="W188" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="X188" t="inlineStr">
+        <is>
+          <t>AFARE</t>
+        </is>
+      </c>
+      <c r="Y188" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z188" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:16:56</t>
+        </is>
+      </c>
+      <c r="AA188" t="n">
+        <v>2920722919</v>
+      </c>
+      <c r="AB188" t="inlineStr">
+        <is>
+          <t>Rid:domestic_1011</t>
+        </is>
+      </c>
+      <c r="AC188" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AD188" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AE188" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>2920745563</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>xss.trade.qunar.com</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>1</v>
+      </c>
+      <c r="D189" t="n">
+        <v>0</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I189" t="n">
+        <v>0</v>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>1970-01-01</t>
+        </is>
+      </c>
+      <c r="K189" t="n">
+        <v>-62170185600000</v>
+      </c>
+      <c r="L189" t="inlineStr"/>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr"/>
+      <c r="O189" t="n">
+        <v>-2</v>
+      </c>
+      <c r="P189" t="inlineStr"/>
+      <c r="Q189" t="n">
+        <v>1</v>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="S189" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:47:30</t>
+        </is>
+      </c>
+      <c r="T189" t="n">
+        <v>1</v>
+      </c>
+      <c r="U189" t="n">
+        <v>0</v>
+      </c>
+      <c r="V189" t="n">
+        <v>0</v>
+      </c>
+      <c r="W189" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="X189" t="inlineStr">
+        <is>
+          <t>AFARE</t>
+        </is>
+      </c>
+      <c r="Y189" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z189" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:17:30</t>
+        </is>
+      </c>
+      <c r="AA189" t="n">
+        <v>2920745563</v>
+      </c>
+      <c r="AB189" t="inlineStr">
+        <is>
+          <t>Rid:domestic_6001</t>
+        </is>
+      </c>
+      <c r="AC189" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AD189" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AE189" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>2920841347</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>xss.trade.qunar.com</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>1</v>
+      </c>
+      <c r="D190" t="n">
+        <v>0</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I190" t="n">
+        <v>0</v>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>1970-01-01</t>
+        </is>
+      </c>
+      <c r="K190" t="n">
+        <v>-62170185600000</v>
+      </c>
+      <c r="L190" t="inlineStr"/>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>2026-09-29 09:21:13</t>
+        </is>
+      </c>
+      <c r="O190" t="n">
+        <v>-2</v>
+      </c>
+      <c r="P190" t="inlineStr"/>
+      <c r="Q190" t="n">
+        <v>1</v>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="S190" t="inlineStr">
+        <is>
+          <t>2026-09-29 17:21:13</t>
+        </is>
+      </c>
+      <c r="T190" t="n">
+        <v>1</v>
+      </c>
+      <c r="U190" t="n">
+        <v>0</v>
+      </c>
+      <c r="V190" t="n">
+        <v>0</v>
+      </c>
+      <c r="W190" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="X190" t="inlineStr">
+        <is>
+          <t>AFARE</t>
+        </is>
+      </c>
+      <c r="Y190" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z190" t="inlineStr">
+        <is>
+          <t>2026-09-29 17:51:13</t>
+        </is>
+      </c>
+      <c r="AA190" t="inlineStr">
+        <is>
+          <t>2920841347</t>
+        </is>
+      </c>
+      <c r="AB190" t="inlineStr">
+        <is>
+          <t>Rid:domestic_6001</t>
+        </is>
+      </c>
+      <c r="AC190" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AD190" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AE190" t="inlineStr">
         <is>
           <t>*</t>
         </is>

</xml_diff>

<commit_message>
data: sync PC-server-0148 2026-10-24 17:26
</commit_message>
<xml_diff>
--- a/data/去哪儿xss.xlsx
+++ b/data/去哪儿xss.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE314"/>
+  <dimension ref="A1:AE315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38185,11 +38185,7 @@
           <t>*</t>
         </is>
       </c>
-      <c r="N314" t="inlineStr">
-        <is>
-          <t>2026-10-23 04:15:52</t>
-        </is>
-      </c>
+      <c r="N314" t="inlineStr"/>
       <c r="O314" t="n">
         <v>-2</v>
       </c>
@@ -38234,10 +38230,8 @@
           <t>2026-10-23 12:45:52</t>
         </is>
       </c>
-      <c r="AA314" t="inlineStr">
-        <is>
-          <t>2927751352</t>
-        </is>
+      <c r="AA314" t="n">
+        <v>2927751352</v>
       </c>
       <c r="AB314" t="inlineStr">
         <is>
@@ -38255,6 +38249,133 @@
         </is>
       </c>
       <c r="AE314" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>2927941063</v>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>xss.trade.qunar.com</t>
+        </is>
+      </c>
+      <c r="C315" t="n">
+        <v>1</v>
+      </c>
+      <c r="D315" t="n">
+        <v>0</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I315" t="n">
+        <v>0</v>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>1970-01-01</t>
+        </is>
+      </c>
+      <c r="K315" t="n">
+        <v>-62170185600000</v>
+      </c>
+      <c r="L315" t="inlineStr"/>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="N315" t="inlineStr">
+        <is>
+          <t>2026-10-24 01:13:18</t>
+        </is>
+      </c>
+      <c r="O315" t="n">
+        <v>-2</v>
+      </c>
+      <c r="P315" t="inlineStr"/>
+      <c r="Q315" t="n">
+        <v>1</v>
+      </c>
+      <c r="R315" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="S315" t="inlineStr">
+        <is>
+          <t>2026-10-24 09:13:18</t>
+        </is>
+      </c>
+      <c r="T315" t="n">
+        <v>1</v>
+      </c>
+      <c r="U315" t="n">
+        <v>0</v>
+      </c>
+      <c r="V315" t="n">
+        <v>0</v>
+      </c>
+      <c r="W315" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="X315" t="inlineStr">
+        <is>
+          <t>AFARE</t>
+        </is>
+      </c>
+      <c r="Y315" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z315" t="inlineStr">
+        <is>
+          <t>2026-10-24 09:43:18</t>
+        </is>
+      </c>
+      <c r="AA315" t="inlineStr">
+        <is>
+          <t>2927941063</t>
+        </is>
+      </c>
+      <c r="AB315" t="inlineStr">
+        <is>
+          <t>Rid:domestic_7001</t>
+        </is>
+      </c>
+      <c r="AC315" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AD315" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="AE315" t="inlineStr">
         <is>
           <t>*</t>
         </is>

</xml_diff>